<commit_message>
feature: add settings.set_accept_empty_as_zero(True) #7
</commit_message>
<xml_diff>
--- a/examples/files/Beispiel.xlsx
+++ b/examples/files/Beispiel.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="680" windowWidth="34200" windowHeight="19380" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Tabelle" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Varianten" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tabelle" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Varianten" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="181029" fullCalcOnLoad="1"/>
@@ -999,7 +999,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D3" t="n">
         <v>2</v>

</xml_diff>